<commit_message>
Fixes frequency response for Voltage measurement
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_D_Inverter/Rev03/BOM/UZ_D_Inverter.xlsx
+++ b/Project Outputs for UZ_D_Inverter/Rev03/BOM/UZ_D_Inverter.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_d_inverter\Project Outputs for UZ_D_Inverter\Rev03\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9022121B-E747-4F0A-9576-6558B0907E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{205D51BE-683C-49BF-B2D8-01DC8C4BFF6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3672" yWindow="-16824" windowWidth="23040" windowHeight="12060" xr2:uid="{A4BB290D-7D8A-4A4C-B39F-C0F291104032}"/>
+    <workbookView xWindow="3456" yWindow="3456" windowWidth="23040" windowHeight="12120" xr2:uid="{23FA5094-82E4-48B4-8857-79C6470B7844}"/>
   </bookViews>
   <sheets>
     <sheet name="UZ_D_Inverter" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="223">
   <si>
     <t>Designator</t>
   </si>
@@ -107,7 +107,7 @@
     <t>10 nF</t>
   </si>
   <si>
-    <t>C11A, C11B, C11C, C12A, C12B, C12C, C15A, C15B, C15C, C16A, C16B, C16C, C50, C51, C55, C56</t>
+    <t>C11A, C11B, C11C, C12A, C12B, C12C, C16A, C16B, C16C, C50, C51, C56</t>
   </si>
   <si>
     <t>Capacitor 0603, 50 VDC, 56 pF, C0G</t>
@@ -125,31 +125,28 @@
     <t>56 pF</t>
   </si>
   <si>
-    <t>C13A, C13B, C13C, C53</t>
-  </si>
-  <si>
-    <t>Capacitor 0805, 100 VDC, 4.7 nF, C0G</t>
-  </si>
-  <si>
-    <t>80-C0805C472F1GEAULR</t>
+    <t>C14A, C14B, C14C, C54</t>
+  </si>
+  <si>
+    <t>Capacitor 0805, 100 VDC, 0.01 µF, C0G</t>
+  </si>
+  <si>
+    <t>80-C0805C103F1GECAUT</t>
   </si>
   <si>
     <t>C_0805</t>
   </si>
   <si>
-    <t>4.7 nF</t>
-  </si>
-  <si>
-    <t>C14A, C14B, C14C, C54</t>
-  </si>
-  <si>
-    <t>Capacitor 0805, 100 VDC, 3.3 nF, C0G</t>
-  </si>
-  <si>
-    <t>80-C0805C332F1G</t>
-  </si>
-  <si>
-    <t>3.3 nF</t>
+    <t>0.01 µF</t>
+  </si>
+  <si>
+    <t>C15A, C15B, C15C, C55</t>
+  </si>
+  <si>
+    <t>Capacitor 0603, 25 VDC, 0.01 µF, C0G</t>
+  </si>
+  <si>
+    <t>80-C0603C103F3GEC</t>
   </si>
   <si>
     <t>C17A, C17B, C17C, C19A, C19B, C19C, C20A, C20B, C20C, C22A, C22B, C22C, C23A, C23B, C23C, C24A, C24B, C24C, C57, C58, C59, C60, C66A, C66B, C66C, C67A, C67B, C67C, C68A, C68B, C68C, C69A, C69B, C69C, C72A, C72B, C72C, C73A, C73B, C73C, C80, C80A, C80B, C80C, C81A, C81B, C81C, C82A, C82B, C82C, C83A, C83B, C83C, C84, C99</t>
@@ -350,6 +347,21 @@
     <t>PCB mount 4mm jack, Black	FCR7350B, 1000V, 24A</t>
   </si>
   <si>
+    <t>J8</t>
+  </si>
+  <si>
+    <t>8 Pin</t>
+  </si>
+  <si>
+    <t>571-103741-8</t>
+  </si>
+  <si>
+    <t>Pin Header</t>
+  </si>
+  <si>
+    <t>HDR1X8</t>
+  </si>
+  <si>
     <t>L1A, L1B, L1C, L2A, L2B, L2C, L3A, L3B, L3C, L4A, L4B, L4C, L5A, L5B, L5C, L6, L7, L8, L9A, L9B, L9C, L10A, L10B, L10C, L12</t>
   </si>
   <si>
@@ -407,7 +419,7 @@
     <t>100V, 97A</t>
   </si>
   <si>
-    <t>R1, R5, R9</t>
+    <t>R1, R2, R3, R5, R9</t>
   </si>
   <si>
     <t>SMD resistor E24 series</t>
@@ -684,6 +696,18 @@
   </si>
   <si>
     <t>SOT95P280X145-6N</t>
+  </si>
+  <si>
+    <t>X2A, X2B, X2C, X3A, X3B, X3C</t>
+  </si>
+  <si>
+    <t>Pin Header, 2.54mm, 1 Pin</t>
+  </si>
+  <si>
+    <t>571-4-103327-3</t>
+  </si>
+  <si>
+    <t>1_Pin_Header</t>
   </si>
 </sst>
 </file>
@@ -1059,18 +1083,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7362835-B2FD-434F-8CEB-EE623EB6FC9A}">
-  <dimension ref="A1:J47"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B55FD43-E243-4864-AC2F-591BFCD48C6C}">
+  <dimension ref="A1:J49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="12.36328125" customWidth="1"/>
-    <col min="3" max="3" width="43.6328125" customWidth="1"/>
-    <col min="4" max="4" width="9" customWidth="1"/>
-    <col min="5" max="10" width="16" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="53" customWidth="1"/>
+    <col min="4" max="4" width="9.21875" customWidth="1"/>
+    <col min="5" max="10" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1102,7 +1126,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>10</v>
       </c>
@@ -1134,7 +1158,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -1166,7 +1190,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>22</v>
       </c>
@@ -1186,7 +1210,7 @@
         <v>15</v>
       </c>
       <c r="G4" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>16</v>
@@ -1198,7 +1222,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>28</v>
       </c>
@@ -1230,7 +1254,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>33</v>
       </c>
@@ -1247,7 +1271,7 @@
         <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="G6" s="1">
         <v>4</v>
@@ -1259,18 +1283,18 @@
         <v>13</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>13</v>
@@ -1291,27 +1315,27 @@
         <v>13</v>
       </c>
       <c r="J7" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="G8" s="1">
         <v>10</v>
@@ -1323,18 +1347,18 @@
         <v>13</v>
       </c>
       <c r="J8" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>13</v>
@@ -1355,18 +1379,18 @@
         <v>13</v>
       </c>
       <c r="J9" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="B10" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>25</v>
@@ -1387,27 +1411,27 @@
         <v>26</v>
       </c>
       <c r="J10" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="B11" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>56</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="G11" s="1">
         <v>10</v>
@@ -1419,27 +1443,27 @@
         <v>13</v>
       </c>
       <c r="J11" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="B12" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="F12" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G12" s="1">
         <v>1</v>
@@ -1448,28 +1472,28 @@
         <v>16</v>
       </c>
       <c r="I12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="B13" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>69</v>
-      </c>
       <c r="E13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G13" s="1">
         <v>1</v>
@@ -1478,28 +1502,28 @@
         <v>16</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="C14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="E14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G14" s="1">
         <v>1</v>
@@ -1508,28 +1532,28 @@
         <v>16</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>77</v>
       </c>
       <c r="G15" s="1">
         <v>3</v>
@@ -1541,27 +1565,27 @@
         <v>13</v>
       </c>
       <c r="J15" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="B16" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>82</v>
       </c>
       <c r="G16" s="1">
         <v>2</v>
@@ -1576,184 +1600,178 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="F17" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>88</v>
       </c>
       <c r="G17" s="1">
         <v>1</v>
       </c>
       <c r="H17" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="I17" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="J17" s="2" t="s">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="B18" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G18" s="1">
         <v>1</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J18" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="B19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="2" t="s">
-        <v>101</v>
-      </c>
       <c r="F19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G19" s="1">
         <v>3</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J19" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="1"/>
+      <c r="E20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E20" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="1">
+        <v>1</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G20" s="1">
+      <c r="B21" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G21" s="1">
         <v>25</v>
       </c>
-      <c r="H20" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="H21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F21" s="2" t="s">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="G21" s="1">
-        <v>6</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J21" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="E22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>119</v>
       </c>
       <c r="G22" s="1">
         <v>6</v>
@@ -1762,152 +1780,156 @@
         <v>16</v>
       </c>
       <c r="I22" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="J22" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="E23" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F23" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="G23" s="1">
+        <v>6</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F23" s="2" t="s">
+      <c r="J23" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="G23" s="1">
-        <v>3</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J23" s="2" t="s">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>123</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>128</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G24" s="1">
+        <v>5</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G25" s="1">
         <v>19</v>
       </c>
-      <c r="H24" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J24" s="2" t="s">
+      <c r="H25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G25" s="1">
+      <c r="G26" s="1">
         <v>7</v>
       </c>
-      <c r="H25" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G26" s="1">
-        <v>1</v>
-      </c>
       <c r="H26" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="I26" s="1"/>
+      <c r="I26" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="J26" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G27" s="1">
         <v>1</v>
@@ -1917,62 +1939,58 @@
       </c>
       <c r="I27" s="1"/>
       <c r="J27" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D28" s="1"/>
       <c r="E28" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F28" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G28" s="1">
+        <v>1</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" s="1"/>
+      <c r="J28" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="G28" s="1">
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="G29" s="1">
         <v>4</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G29" s="1">
-        <v>12</v>
       </c>
       <c r="H29" s="2" t="s">
         <v>16</v>
@@ -1984,24 +2002,24 @@
         <v>147</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>148</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G30" s="1">
         <v>12</v>
@@ -2010,18 +2028,18 @@
         <v>16</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>153</v>
@@ -2033,10 +2051,10 @@
         <v>14</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G31" s="1">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>16</v>
@@ -2048,7 +2066,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>155</v>
       </c>
@@ -2059,13 +2077,13 @@
         <v>157</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G32" s="1">
         <v>16</v>
@@ -2074,31 +2092,31 @@
         <v>16</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="J32" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>125</v>
-      </c>
       <c r="G33" s="1">
         <v>16</v>
       </c>
@@ -2109,15 +2127,15 @@
         <v>13</v>
       </c>
       <c r="J33" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>162</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>163</v>
@@ -2129,10 +2147,10 @@
         <v>14</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G34" s="1">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>16</v>
@@ -2144,15 +2162,15 @@
         <v>164</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>165</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>13</v>
@@ -2161,7 +2179,7 @@
         <v>14</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G35" s="1">
         <v>6</v>
@@ -2173,18 +2191,18 @@
         <v>13</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>152</v>
+        <v>166</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>13</v>
@@ -2193,7 +2211,7 @@
         <v>14</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>170</v>
+        <v>129</v>
       </c>
       <c r="G36" s="1">
         <v>6</v>
@@ -2208,12 +2226,12 @@
         <v>171</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>172</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>173</v>
@@ -2225,7 +2243,7 @@
         <v>14</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>125</v>
+        <v>174</v>
       </c>
       <c r="G37" s="1">
         <v>6</v>
@@ -2237,18 +2255,18 @@
         <v>13</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D38" s="2" t="s">
         <v>13</v>
@@ -2257,7 +2275,7 @@
         <v>14</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G38" s="1">
         <v>6</v>
@@ -2269,18 +2287,18 @@
         <v>13</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>123</v>
+        <v>166</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D39" s="2" t="s">
         <v>13</v>
@@ -2289,42 +2307,42 @@
         <v>14</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="G39" s="1">
+        <v>6</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G40" s="1">
         <v>8</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A40" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="G40" s="1">
-        <v>6</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>16</v>
@@ -2336,39 +2354,39 @@
         <v>184</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>185</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="D41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D41" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F41" s="2" t="s">
+      <c r="G41" s="1">
+        <v>6</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J41" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="G41" s="1">
-        <v>5</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>189</v>
       </c>
@@ -2382,25 +2400,25 @@
         <v>13</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>192</v>
       </c>
       <c r="G42" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>16</v>
+        <v>191</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>13</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>193</v>
       </c>
@@ -2411,74 +2429,74 @@
         <v>195</v>
       </c>
       <c r="D43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F43" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="E43" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F43" s="2" t="s">
+      <c r="G43" s="1">
+        <v>4</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="G43" s="1">
+      <c r="B44" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="G44" s="1">
         <v>8</v>
       </c>
-      <c r="H43" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I43" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J43" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A44" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="E44" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F44" s="2" t="s">
+      <c r="H44" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="G44" s="1">
-        <v>6</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="J44" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="C45" s="2" t="s">
+      <c r="D45" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="E45" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>206</v>
@@ -2490,13 +2508,13 @@
         <v>16</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>13</v>
+        <v>88</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>207</v>
       </c>
@@ -2510,13 +2528,13 @@
         <v>13</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>210</v>
       </c>
       <c r="G46" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H46" s="2" t="s">
         <v>16</v>
@@ -2528,7 +2546,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>211</v>
       </c>
@@ -2538,24 +2556,88 @@
       <c r="C47" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="D47" s="1"/>
+      <c r="D47" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="E47" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>214</v>
       </c>
       <c r="G47" s="1">
+        <v>3</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D48" s="1"/>
+      <c r="E48" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G48" s="1">
         <v>1</v>
       </c>
-      <c r="H47" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" s="1"/>
-      <c r="J47" s="1"/>
+      <c r="H48" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" s="1"/>
+      <c r="J48" s="1"/>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G49" s="1">
+        <v>6</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>